<commit_message>
fix 3.3 thêm hợp đồng bằng file
</commit_message>
<xml_diff>
--- a/static/uploads/mau/nhaphophong/taohopdong.xlsx
+++ b/static/uploads/mau/nhaphophong/taohopdong.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26327"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Khanh\Desktop\HRM\static\uploads\mau\nhaphophong\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Code\HRM\static\uploads\mau\nhaphophong\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BBE09B31-07DC-4A48-B45B-4ADA346F0B22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2CB769E-03A1-4D96-8E2D-66BD80693317}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{EF705DD9-3C65-4824-9431-C7CE35B9AF6D}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="15600" windowHeight="11040" xr2:uid="{EF705DD9-3C65-4824-9431-C7CE35B9AF6D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="35">
   <si>
     <t>Mã công ty</t>
   </si>
@@ -125,6 +125,12 @@
   </si>
   <si>
     <t>Phụ lục hợp đồng</t>
+  </si>
+  <si>
+    <t>Nơi cấp</t>
+  </si>
+  <si>
+    <t>Cục cảnh sát</t>
   </si>
 </sst>
 </file>
@@ -132,8 +138,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
-    <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="164" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="165" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
@@ -207,7 +213,7 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -220,10 +226,10 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="2" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -254,9 +260,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -294,7 +300,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -400,7 +406,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -542,7 +548,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -550,30 +556,31 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F3B7851E-53E1-4A92-8724-271B72814170}">
-  <dimension ref="A1:R43"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:S43"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="10.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.5546875" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="6" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.44140625" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="9" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="42.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="51.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.140625" style="7" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="7.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="26.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="40.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="18.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="7.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="14.85546875" style="5" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="9.28515625" style="5" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="15.85546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="16.28515625" style="3" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="42.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="51.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.109375" style="7" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.109375" style="1" customWidth="1"/>
+    <col min="11" max="11" width="7.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="26.109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="40.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="18.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="7.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="14.88671875" style="5" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="9.33203125" style="5" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="15.88671875" style="3" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="16.33203125" style="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -602,34 +609,37 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="K1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="L1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="M1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="N1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="2" t="s">
+      <c r="O1" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="4" t="s">
+      <c r="P1" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="4" t="s">
+      <c r="Q1" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="8" t="s">
+      <c r="R1" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="R1" s="8" t="s">
+      <c r="S1" s="8" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>18</v>
       </c>
@@ -658,401 +668,445 @@
         <v>44311</v>
       </c>
       <c r="J2" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="K2" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="K2" s="1" t="s">
+      <c r="L2" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="L2" s="1" t="s">
+      <c r="M2" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="M2" s="3" t="s">
+      <c r="N2" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="N2" s="1" t="s">
+      <c r="O2" s="1" t="s">
         <v>21</v>
-      </c>
-      <c r="O2" s="5">
-        <v>0</v>
       </c>
       <c r="P2" s="5">
         <v>0</v>
       </c>
-      <c r="Q2" s="3">
+      <c r="Q2" s="5">
+        <v>0</v>
+      </c>
+      <c r="R2" s="3">
         <v>45481</v>
       </c>
-      <c r="R2" s="3">
+      <c r="S2" s="3">
         <v>45845</v>
       </c>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:19" x14ac:dyDescent="0.3">
       <c r="E3" s="3"/>
       <c r="F3" s="3"/>
       <c r="G3" s="3"/>
       <c r="H3" s="3"/>
       <c r="I3" s="3"/>
       <c r="J3" s="3"/>
-      <c r="M3" s="3"/>
-    </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="K3" s="3"/>
+      <c r="N3" s="3"/>
+    </row>
+    <row r="4" spans="1:19" x14ac:dyDescent="0.3">
       <c r="E4" s="3"/>
       <c r="F4" s="3"/>
       <c r="G4" s="3"/>
       <c r="H4" s="3"/>
       <c r="I4" s="3"/>
       <c r="J4" s="3"/>
-      <c r="M4" s="3"/>
-    </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="K4" s="3"/>
+      <c r="N4" s="3"/>
+    </row>
+    <row r="5" spans="1:19" x14ac:dyDescent="0.3">
       <c r="E5" s="3"/>
       <c r="F5" s="3"/>
       <c r="G5" s="3"/>
       <c r="H5" s="3"/>
       <c r="I5" s="3"/>
       <c r="J5" s="3"/>
-      <c r="M5" s="3"/>
-    </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="K5" s="3"/>
+      <c r="N5" s="3"/>
+    </row>
+    <row r="6" spans="1:19" x14ac:dyDescent="0.3">
       <c r="E6" s="3"/>
       <c r="F6" s="3"/>
       <c r="G6" s="3"/>
       <c r="H6" s="3"/>
       <c r="I6" s="3"/>
       <c r="J6" s="3"/>
-      <c r="M6" s="3"/>
-    </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="K6" s="3"/>
+      <c r="N6" s="3"/>
+    </row>
+    <row r="7" spans="1:19" x14ac:dyDescent="0.3">
       <c r="E7" s="3"/>
       <c r="F7" s="3"/>
       <c r="G7" s="3"/>
       <c r="H7" s="3"/>
       <c r="I7" s="3"/>
       <c r="J7" s="3"/>
-      <c r="M7" s="3"/>
-    </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="K7" s="3"/>
+      <c r="N7" s="3"/>
+    </row>
+    <row r="8" spans="1:19" x14ac:dyDescent="0.3">
       <c r="E8" s="3"/>
       <c r="F8" s="3"/>
       <c r="G8" s="3"/>
       <c r="H8" s="3"/>
       <c r="I8" s="3"/>
       <c r="J8" s="3"/>
-      <c r="M8" s="3"/>
-    </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="K8" s="3"/>
+      <c r="N8" s="3"/>
+    </row>
+    <row r="9" spans="1:19" x14ac:dyDescent="0.3">
       <c r="E9" s="3"/>
       <c r="F9" s="3"/>
       <c r="G9" s="3"/>
       <c r="H9" s="3"/>
       <c r="I9" s="3"/>
       <c r="J9" s="3"/>
-      <c r="M9" s="3"/>
-    </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="K9" s="3"/>
+      <c r="N9" s="3"/>
+    </row>
+    <row r="10" spans="1:19" x14ac:dyDescent="0.3">
       <c r="E10" s="3"/>
       <c r="F10" s="3"/>
       <c r="G10" s="3"/>
       <c r="H10" s="3"/>
       <c r="I10" s="3"/>
       <c r="J10" s="3"/>
-      <c r="M10" s="3"/>
-    </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="K10" s="3"/>
+      <c r="N10" s="3"/>
+    </row>
+    <row r="11" spans="1:19" x14ac:dyDescent="0.3">
       <c r="E11" s="3"/>
       <c r="F11" s="3"/>
       <c r="G11" s="3"/>
       <c r="H11" s="3"/>
       <c r="I11" s="3"/>
       <c r="J11" s="3"/>
-      <c r="M11" s="3"/>
-    </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="K11" s="3"/>
+      <c r="N11" s="3"/>
+    </row>
+    <row r="12" spans="1:19" x14ac:dyDescent="0.3">
       <c r="E12" s="3"/>
       <c r="F12" s="3"/>
       <c r="G12" s="3"/>
       <c r="H12" s="3"/>
       <c r="I12" s="3"/>
       <c r="J12" s="3"/>
-      <c r="M12" s="3"/>
-    </row>
-    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="K12" s="3"/>
+      <c r="N12" s="3"/>
+    </row>
+    <row r="13" spans="1:19" x14ac:dyDescent="0.3">
       <c r="E13" s="3"/>
       <c r="F13" s="3"/>
       <c r="G13" s="3"/>
       <c r="H13" s="3"/>
       <c r="I13" s="3"/>
       <c r="J13" s="3"/>
-      <c r="M13" s="3"/>
-    </row>
-    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="K13" s="3"/>
+      <c r="N13" s="3"/>
+    </row>
+    <row r="14" spans="1:19" x14ac:dyDescent="0.3">
       <c r="E14" s="3"/>
       <c r="F14" s="3"/>
       <c r="G14" s="3"/>
       <c r="H14" s="3"/>
       <c r="I14" s="3"/>
       <c r="J14" s="3"/>
-      <c r="M14" s="3"/>
-    </row>
-    <row r="15" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="K14" s="3"/>
+      <c r="N14" s="3"/>
+    </row>
+    <row r="15" spans="1:19" x14ac:dyDescent="0.3">
       <c r="E15" s="3"/>
       <c r="F15" s="3"/>
       <c r="G15" s="3"/>
       <c r="H15" s="3"/>
       <c r="I15" s="3"/>
       <c r="J15" s="3"/>
-      <c r="M15" s="3"/>
-    </row>
-    <row r="16" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="K15" s="3"/>
+      <c r="N15" s="3"/>
+    </row>
+    <row r="16" spans="1:19" x14ac:dyDescent="0.3">
       <c r="E16" s="3"/>
       <c r="F16" s="3"/>
       <c r="G16" s="3"/>
       <c r="H16" s="3"/>
       <c r="I16" s="3"/>
       <c r="J16" s="3"/>
-      <c r="M16" s="3"/>
-    </row>
-    <row r="17" spans="5:13" x14ac:dyDescent="0.25">
+      <c r="K16" s="3"/>
+      <c r="N16" s="3"/>
+    </row>
+    <row r="17" spans="5:14" x14ac:dyDescent="0.3">
       <c r="E17" s="3"/>
       <c r="F17" s="3"/>
       <c r="G17" s="3"/>
       <c r="H17" s="3"/>
       <c r="I17" s="3"/>
       <c r="J17" s="3"/>
-      <c r="M17" s="3"/>
-    </row>
-    <row r="18" spans="5:13" x14ac:dyDescent="0.25">
+      <c r="K17" s="3"/>
+      <c r="N17" s="3"/>
+    </row>
+    <row r="18" spans="5:14" x14ac:dyDescent="0.3">
       <c r="E18" s="3"/>
       <c r="F18" s="3"/>
       <c r="G18" s="3"/>
       <c r="H18" s="3"/>
       <c r="I18" s="3"/>
       <c r="J18" s="3"/>
-      <c r="M18" s="3"/>
-    </row>
-    <row r="19" spans="5:13" x14ac:dyDescent="0.25">
+      <c r="K18" s="3"/>
+      <c r="N18" s="3"/>
+    </row>
+    <row r="19" spans="5:14" x14ac:dyDescent="0.3">
       <c r="E19" s="3"/>
       <c r="F19" s="3"/>
       <c r="G19" s="3"/>
       <c r="H19" s="3"/>
       <c r="I19" s="3"/>
       <c r="J19" s="3"/>
-      <c r="M19" s="3"/>
-    </row>
-    <row r="20" spans="5:13" x14ac:dyDescent="0.25">
+      <c r="K19" s="3"/>
+      <c r="N19" s="3"/>
+    </row>
+    <row r="20" spans="5:14" x14ac:dyDescent="0.3">
       <c r="E20" s="3"/>
       <c r="F20" s="3"/>
       <c r="G20" s="3"/>
       <c r="H20" s="3"/>
       <c r="I20" s="3"/>
       <c r="J20" s="3"/>
-      <c r="M20" s="3"/>
-    </row>
-    <row r="21" spans="5:13" x14ac:dyDescent="0.25">
+      <c r="K20" s="3"/>
+      <c r="N20" s="3"/>
+    </row>
+    <row r="21" spans="5:14" x14ac:dyDescent="0.3">
       <c r="E21" s="3"/>
       <c r="F21" s="3"/>
       <c r="G21" s="3"/>
       <c r="H21" s="3"/>
       <c r="I21" s="3"/>
       <c r="J21" s="3"/>
-      <c r="M21" s="3"/>
-    </row>
-    <row r="22" spans="5:13" x14ac:dyDescent="0.25">
+      <c r="K21" s="3"/>
+      <c r="N21" s="3"/>
+    </row>
+    <row r="22" spans="5:14" x14ac:dyDescent="0.3">
       <c r="E22" s="3"/>
       <c r="F22" s="3"/>
       <c r="G22" s="3"/>
       <c r="H22" s="3"/>
       <c r="I22" s="3"/>
       <c r="J22" s="3"/>
-      <c r="M22" s="3"/>
-    </row>
-    <row r="23" spans="5:13" x14ac:dyDescent="0.25">
+      <c r="K22" s="3"/>
+      <c r="N22" s="3"/>
+    </row>
+    <row r="23" spans="5:14" x14ac:dyDescent="0.3">
       <c r="E23" s="3"/>
       <c r="F23" s="3"/>
       <c r="G23" s="3"/>
       <c r="H23" s="3"/>
       <c r="I23" s="3"/>
       <c r="J23" s="3"/>
-      <c r="M23" s="3"/>
-    </row>
-    <row r="24" spans="5:13" x14ac:dyDescent="0.25">
+      <c r="K23" s="3"/>
+      <c r="N23" s="3"/>
+    </row>
+    <row r="24" spans="5:14" x14ac:dyDescent="0.3">
       <c r="E24" s="3"/>
       <c r="F24" s="3"/>
       <c r="G24" s="3"/>
       <c r="H24" s="3"/>
       <c r="I24" s="3"/>
       <c r="J24" s="3"/>
-      <c r="M24" s="3"/>
-    </row>
-    <row r="25" spans="5:13" x14ac:dyDescent="0.25">
+      <c r="K24" s="3"/>
+      <c r="N24" s="3"/>
+    </row>
+    <row r="25" spans="5:14" x14ac:dyDescent="0.3">
       <c r="E25" s="3"/>
       <c r="F25" s="3"/>
       <c r="G25" s="3"/>
       <c r="H25" s="3"/>
       <c r="I25" s="3"/>
       <c r="J25" s="3"/>
-      <c r="M25" s="3"/>
-    </row>
-    <row r="26" spans="5:13" x14ac:dyDescent="0.25">
+      <c r="K25" s="3"/>
+      <c r="N25" s="3"/>
+    </row>
+    <row r="26" spans="5:14" x14ac:dyDescent="0.3">
       <c r="E26" s="3"/>
       <c r="F26" s="3"/>
       <c r="G26" s="3"/>
       <c r="H26" s="3"/>
       <c r="I26" s="3"/>
       <c r="J26" s="3"/>
-      <c r="M26" s="3"/>
-    </row>
-    <row r="27" spans="5:13" x14ac:dyDescent="0.25">
+      <c r="K26" s="3"/>
+      <c r="N26" s="3"/>
+    </row>
+    <row r="27" spans="5:14" x14ac:dyDescent="0.3">
       <c r="E27" s="3"/>
       <c r="F27" s="3"/>
       <c r="G27" s="3"/>
       <c r="H27" s="3"/>
       <c r="I27" s="3"/>
       <c r="J27" s="3"/>
-      <c r="M27" s="3"/>
-    </row>
-    <row r="28" spans="5:13" x14ac:dyDescent="0.25">
+      <c r="K27" s="3"/>
+      <c r="N27" s="3"/>
+    </row>
+    <row r="28" spans="5:14" x14ac:dyDescent="0.3">
       <c r="E28" s="3"/>
       <c r="F28" s="3"/>
       <c r="G28" s="3"/>
       <c r="H28" s="3"/>
       <c r="I28" s="3"/>
       <c r="J28" s="3"/>
-      <c r="M28" s="3"/>
-    </row>
-    <row r="29" spans="5:13" x14ac:dyDescent="0.25">
+      <c r="K28" s="3"/>
+      <c r="N28" s="3"/>
+    </row>
+    <row r="29" spans="5:14" x14ac:dyDescent="0.3">
       <c r="E29" s="3"/>
       <c r="F29" s="3"/>
       <c r="G29" s="3"/>
       <c r="H29" s="3"/>
       <c r="I29" s="3"/>
       <c r="J29" s="3"/>
-      <c r="M29" s="3"/>
-    </row>
-    <row r="30" spans="5:13" x14ac:dyDescent="0.25">
+      <c r="K29" s="3"/>
+      <c r="N29" s="3"/>
+    </row>
+    <row r="30" spans="5:14" x14ac:dyDescent="0.3">
       <c r="E30" s="3"/>
       <c r="F30" s="3"/>
       <c r="G30" s="3"/>
       <c r="H30" s="3"/>
       <c r="I30" s="3"/>
       <c r="J30" s="3"/>
-      <c r="M30" s="3"/>
-    </row>
-    <row r="31" spans="5:13" x14ac:dyDescent="0.25">
+      <c r="K30" s="3"/>
+      <c r="N30" s="3"/>
+    </row>
+    <row r="31" spans="5:14" x14ac:dyDescent="0.3">
       <c r="E31" s="3"/>
       <c r="F31" s="3"/>
       <c r="G31" s="3"/>
       <c r="H31" s="3"/>
       <c r="I31" s="3"/>
       <c r="J31" s="3"/>
-      <c r="M31" s="3"/>
-    </row>
-    <row r="32" spans="5:13" x14ac:dyDescent="0.25">
+      <c r="K31" s="3"/>
+      <c r="N31" s="3"/>
+    </row>
+    <row r="32" spans="5:14" x14ac:dyDescent="0.3">
       <c r="E32" s="3"/>
       <c r="F32" s="3"/>
       <c r="G32" s="3"/>
       <c r="H32" s="3"/>
       <c r="I32" s="3"/>
       <c r="J32" s="3"/>
-      <c r="M32" s="3"/>
-    </row>
-    <row r="33" spans="5:13" x14ac:dyDescent="0.25">
+      <c r="K32" s="3"/>
+      <c r="N32" s="3"/>
+    </row>
+    <row r="33" spans="5:14" x14ac:dyDescent="0.3">
       <c r="E33" s="3"/>
       <c r="F33" s="3"/>
       <c r="G33" s="3"/>
       <c r="H33" s="3"/>
       <c r="I33" s="3"/>
       <c r="J33" s="3"/>
-      <c r="M33" s="3"/>
-    </row>
-    <row r="34" spans="5:13" x14ac:dyDescent="0.25">
+      <c r="K33" s="3"/>
+      <c r="N33" s="3"/>
+    </row>
+    <row r="34" spans="5:14" x14ac:dyDescent="0.3">
       <c r="E34" s="3"/>
       <c r="F34" s="3"/>
       <c r="G34" s="3"/>
       <c r="H34" s="3"/>
       <c r="I34" s="3"/>
       <c r="J34" s="3"/>
-      <c r="M34" s="3"/>
-    </row>
-    <row r="35" spans="5:13" x14ac:dyDescent="0.25">
+      <c r="K34" s="3"/>
+      <c r="N34" s="3"/>
+    </row>
+    <row r="35" spans="5:14" x14ac:dyDescent="0.3">
       <c r="E35" s="3"/>
       <c r="F35" s="3"/>
       <c r="G35" s="3"/>
       <c r="H35" s="3"/>
       <c r="I35" s="3"/>
       <c r="J35" s="3"/>
-      <c r="M35" s="3"/>
-    </row>
-    <row r="36" spans="5:13" x14ac:dyDescent="0.25">
+      <c r="K35" s="3"/>
+      <c r="N35" s="3"/>
+    </row>
+    <row r="36" spans="5:14" x14ac:dyDescent="0.3">
       <c r="E36" s="3"/>
       <c r="F36" s="3"/>
       <c r="G36" s="3"/>
       <c r="H36" s="3"/>
       <c r="I36" s="3"/>
       <c r="J36" s="3"/>
-      <c r="M36" s="3"/>
-    </row>
-    <row r="37" spans="5:13" x14ac:dyDescent="0.25">
+      <c r="K36" s="3"/>
+      <c r="N36" s="3"/>
+    </row>
+    <row r="37" spans="5:14" x14ac:dyDescent="0.3">
       <c r="E37" s="3"/>
       <c r="F37" s="3"/>
       <c r="G37" s="3"/>
       <c r="H37" s="3"/>
       <c r="I37" s="3"/>
       <c r="J37" s="3"/>
-      <c r="M37" s="3"/>
-    </row>
-    <row r="38" spans="5:13" x14ac:dyDescent="0.25">
+      <c r="K37" s="3"/>
+      <c r="N37" s="3"/>
+    </row>
+    <row r="38" spans="5:14" x14ac:dyDescent="0.3">
       <c r="E38" s="3"/>
       <c r="F38" s="3"/>
       <c r="G38" s="3"/>
       <c r="H38" s="3"/>
       <c r="I38" s="3"/>
       <c r="J38" s="3"/>
-      <c r="M38" s="3"/>
-    </row>
-    <row r="39" spans="5:13" x14ac:dyDescent="0.25">
+      <c r="K38" s="3"/>
+      <c r="N38" s="3"/>
+    </row>
+    <row r="39" spans="5:14" x14ac:dyDescent="0.3">
       <c r="E39" s="3"/>
       <c r="F39" s="3"/>
       <c r="G39" s="3"/>
       <c r="H39" s="3"/>
       <c r="I39" s="3"/>
       <c r="J39" s="3"/>
-      <c r="M39" s="3"/>
-    </row>
-    <row r="40" spans="5:13" x14ac:dyDescent="0.25">
+      <c r="K39" s="3"/>
+      <c r="N39" s="3"/>
+    </row>
+    <row r="40" spans="5:14" x14ac:dyDescent="0.3">
       <c r="E40" s="3"/>
       <c r="F40" s="3"/>
       <c r="G40" s="3"/>
       <c r="H40" s="3"/>
       <c r="I40" s="3"/>
       <c r="J40" s="3"/>
-      <c r="M40" s="3"/>
-    </row>
-    <row r="41" spans="5:13" x14ac:dyDescent="0.25">
+      <c r="K40" s="3"/>
+      <c r="N40" s="3"/>
+    </row>
+    <row r="41" spans="5:14" x14ac:dyDescent="0.3">
       <c r="E41" s="3"/>
       <c r="F41" s="3"/>
       <c r="G41" s="3"/>
       <c r="H41" s="3"/>
       <c r="I41" s="3"/>
       <c r="J41" s="3"/>
-      <c r="M41" s="3"/>
-    </row>
-    <row r="42" spans="5:13" x14ac:dyDescent="0.25">
+      <c r="K41" s="3"/>
+      <c r="N41" s="3"/>
+    </row>
+    <row r="42" spans="5:14" x14ac:dyDescent="0.3">
       <c r="E42" s="3"/>
       <c r="F42" s="3"/>
       <c r="G42" s="3"/>
       <c r="H42" s="3"/>
       <c r="I42" s="3"/>
       <c r="J42" s="3"/>
-      <c r="M42" s="3"/>
-    </row>
-    <row r="43" spans="5:13" x14ac:dyDescent="0.25">
+      <c r="K42" s="3"/>
+      <c r="N42" s="3"/>
+    </row>
+    <row r="43" spans="5:14" x14ac:dyDescent="0.3">
       <c r="E43" s="3"/>
       <c r="F43" s="3"/>
       <c r="G43" s="3"/>
       <c r="H43" s="3"/>
       <c r="I43" s="3"/>
       <c r="J43" s="3"/>
-      <c r="M43" s="3"/>
+      <c r="K43" s="3"/>
+      <c r="N43" s="3"/>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
@@ -1065,7 +1119,7 @@
           <x14:formula1>
             <xm:f>Sheet2!$A$1:$A$5</xm:f>
           </x14:formula1>
-          <xm:sqref>K2:K43</xm:sqref>
+          <xm:sqref>L2:L43</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -1076,32 +1130,32 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{868B83F7-F680-4D08-9C8D-75A22AF6EB36}">
   <dimension ref="A1:A5"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="27.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="27.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>32</v>
       </c>

</xml_diff>